<commit_message>
Voeg EWS- en Hardheidsclausule-sheets toe met relevantiebeoordeling
Per gevalideerde vraag is beoordeeld (Ja/Mogelijk/Nee, met onderbouwing)
of deze bruikbaar is voor het EWS (vastgoed + financiële cijfers) resp.
de hardheidsclausule (FTE, vastgoedcapaciteit, financiële data).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HjW1Vn1BtW4ztesZ4qiQDe
</commit_message>
<xml_diff>
--- a/Gevalideerde_vragen_Uitwisselprofiel_Zorgkantoren.xlsx
+++ b/Gevalideerde_vragen_Uitwisselprofiel_Zorgkantoren.xlsx
@@ -8,10 +8,14 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gevalideerde vragen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toelichting" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EWS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hardheidsclausule" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toelichting" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gevalideerde vragen'!$A$4:$G$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'EWS'!$A$6:$F$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hardheidsclausule'!$A$6:$F$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,8 +65,25 @@
       <sz val="10"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C6500"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +98,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -106,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,6 +168,33 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3124,7 +3187,4611 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:F73"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>EWS (Early Warning System – Zilveren Kruis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Beoordeling welke gevalideerde vragen uit het Uitwisselprofiel Zorgkantoren mogelijk bruikbaar zijn voor het EWS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>vragen over vastgoed(capaciteit) en financiële cijfers om de financiële stabiliteit van een zorgaanbieder in te schatten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Let op: dit is een inhoudelijke inschatting op basis van de vraagomschrijving, niet een officiële koppeling van Zilveren Kruis/KIK-V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Categorie</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Vraag (gevalideerde vraag)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Relevant?</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Onderbouwing</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Link naar indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het aantal aanwezige wooneenheden?</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Vastgoedcapaciteit: aantal aanwezige/bezette wooneenheden en huisvestingscapaciteit per vestiging.</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>15.2</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het aantal bezette wooneenheden?</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Vastgoedcapaciteit: aantal aanwezige/bezette wooneenheden en huisvestingscapaciteit per vestiging.</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>15.3</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Hoeveel personen kunnen er per vestiging wonen?</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Vastgoedcapaciteit: aantal aanwezige/bezette wooneenheden en huisvestingscapaciteit per vestiging.</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>17.1.1</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal wooneenheden voor intramuraal en VPT geclusterd?</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Geplande toe-/afname van vastgoedcapaciteit (wooneenheden); direct relevant voor inschatting van toekomstige vastgoedpositie.</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>17.1.2</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal wooneenheden voor MPT en VPT niet-geclusterd?</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Geplande toe-/afname van vastgoedcapaciteit (wooneenheden); direct relevant voor inschatting van toekomstige vastgoedpositie.</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>18.1</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (balans / W&amp;V)</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de balans o.b.v. Grootboek?</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>18.2</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (balans / W&amp;V)</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de winst- en verliesrekening o.b.v. Grootboek?</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>19.1</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de DSCR (Debt Service Coverage Ratio)?</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>19.2</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is het werkkapitaal op korte termijn?</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>19.3</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de werkkapitaalratio?</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de quick ratio?</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>19.5</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de current ratio?</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>19.6</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de EBITDA (Earnings Before Interest, Tax, Deprecation and Amortisation)?</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de EBITDA-ratio?</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>19.8</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de cashflow?</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>20.1</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is de solvabiliteitsratio?</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>20.2</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is het weerstandsvermogen?</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>20.3</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is de debt ratio?</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat zijn de reserves?</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is de Reserves-Ratio?</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>21.1</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (rentabiliteit)</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Rentabiliteit - wat is de winstratio?</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>21.2</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (rentabiliteit)</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Rentabiliteit - wat is de REV (Resultaat Eigen Vermogen)?</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>22.1</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (groei)</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>Groei - wat is de omzetgroei?</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>23.1</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (kapitaal)</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Kapitaal - wat is de LTV (Loan to Value)?</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>23.2</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (kapitaal)</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Kapitaal - wat is de net-debt / EBITDA?</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>23.3</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (kapitaal)</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>Kapitaal - wat is de CAPEX (Capital Expenditures)?</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>24.1</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de dekking van vaste activia door lang vermogen?</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>24.2</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de Interest Coverage Ratio (ICR)?</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>24.3</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de verhouding tussen kort en lang vreemd vermogen?</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>24.4</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de verhouding tussen vorderingen en opbrengsten?</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de arbeidsintensiteit PIL &amp; PNIL?</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>24.7</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de arbeidsintensiteit PNIL?</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>24.9</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is verhouding tussen uitbesteed werk en vast personeel?</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>15.4.1</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel cliënten met indicaties zijn er per financieringsstroom?</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>Financieel-gerelateerde omzet-/declaratiedata (gedeclareerde bedragen, Wlz-cliënten per sector/financieringsstroom); geeft context bij de omzet maar is geen kernratio voor financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>15.4.2</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel Wlz-cliënten zijn er per sector?</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>Financieel-gerelateerde omzet-/declaratiedata (gedeclareerde bedragen, Wlz-cliënten per sector/financieringsstroom); geeft context bij de omzet maar is geen kernratio voor financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F41" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>15.4.3</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel Wlz-cliënten met zorgprofiel VV zijn er per leveringsvorm?</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>Financieel-gerelateerde omzet-/declaratiedata (gedeclareerde bedragen, Wlz-cliënten per sector/financieringsstroom); geeft context bij de omzet maar is geen kernratio voor financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F42" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>15.4.4</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het gedeclareerde bedrag per wet?</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>Financieel-gerelateerde omzet-/declaratiedata (gedeclareerde bedragen, Wlz-cliënten per sector/financieringsstroom); geeft context bij de omzet maar is geen kernratio voor financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F43" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>15.4.5</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het gedeclareerde bedrag per zorgsector?</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>Financieel-gerelateerde omzet-/declaratiedata (gedeclareerde bedragen, Wlz-cliënten per sector/financieringsstroom); geeft context bij de omzet maar is geen kernratio voor financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>15.4.6</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het gedeclareerde bedrag binnen Wlz-VV per leveringsvorm?</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>Financieel-gerelateerde omzet-/declaratiedata (gedeclareerde bedragen, Wlz-cliënten per sector/financieringsstroom); geeft context bij de omzet maar is geen kernratio voor financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>17.2.1</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal cliënten voor intramuraal en VPT geclusterd?</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="inlineStr">
+        <is>
+          <t>Geplande cliëntontwikkeling gekoppeld aan de vastgoedplanning; indirect relevant voor de vastgoed-/capaciteitsinschatting, maar zelf geen vastgoed- of financieel gegeven.</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>17.2.2</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal cliënten voor MPT en VPT niet-geclusterd?</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>Geplande cliëntontwikkeling gekoppeld aan de vastgoedplanning; indirect relevant voor de vastgoed-/capaciteitsinschatting, maar zelf geen vastgoed- of financieel gegeven.</t>
+        </is>
+      </c>
+      <c r="F47" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het gemiddeld aantal personeelsleden?</t>
+        </is>
+      </c>
+      <c r="D48" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E48" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F48" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B49" s="17" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het aantal personeelsleden?</t>
+        </is>
+      </c>
+      <c r="D49" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F49" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B50" s="17" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>Hoeveel uren zorggerelateerd personeel wordt ingezet?</t>
+        </is>
+      </c>
+      <c r="D50" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E50" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F50" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="B51" s="17" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>Hoeveel uur zijn er verloond?</t>
+        </is>
+      </c>
+      <c r="D51" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E51" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F51" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>Welk deel van de arbeidsovereenkomsten is voor bepaalde tijd?</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F52" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="B53" s="17" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>Wat is de gemiddelde contractomvang?</t>
+        </is>
+      </c>
+      <c r="D53" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F53" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>Wat is de leeftijdsopbouw van het personeel in loondienst?</t>
+        </is>
+      </c>
+      <c r="D54" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F54" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="B55" s="17" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="inlineStr">
+        <is>
+          <t>Hoe zijn de ingezette uren zorgverleners verdeeld over de kwalificatieniveaus?</t>
+        </is>
+      </c>
+      <c r="D55" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F55" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="B56" s="17" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C56" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het aantal ingezette uren zorgverleners in loondienst per cliënt?</t>
+        </is>
+      </c>
+      <c r="D56" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F56" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="B57" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (PNIL)</t>
+        </is>
+      </c>
+      <c r="C57" s="17" t="inlineStr">
+        <is>
+          <t>Welk deel van de ingezette uren personeel is door PNIL?</t>
+        </is>
+      </c>
+      <c r="D57" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E57" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F57" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="B58" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (PNIL)</t>
+        </is>
+      </c>
+      <c r="C58" s="17" t="inlineStr">
+        <is>
+          <t>Welk deel van de personeelskosten zijn voor PNIL?</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E58" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F58" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (vrijwilligers)</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het aantal vrijwilligers?</t>
+        </is>
+      </c>
+      <c r="D59" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E59" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F59" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="B60" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (BBL)</t>
+        </is>
+      </c>
+      <c r="C60" s="17" t="inlineStr">
+        <is>
+          <t>Hoeveel BBL leerlingen zijn er?</t>
+        </is>
+      </c>
+      <c r="D60" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E60" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F60" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="B61" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het kortdurend ziekteverzuimpercentage excl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E61" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F61" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="B62" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C62" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het kortdurend ziekteverzuimpercentage incl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E62" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F62" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="B63" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het langdurend ziekteverzuimpercentage excl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D63" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E63" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F63" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="B64" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C64" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het langdurend ziekteverzuimpercentage incl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D64" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E64" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F64" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="B65" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C65" s="17" t="inlineStr">
+        <is>
+          <t>Wat is de verzuimfrequentie excl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D65" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E65" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F65" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="B66" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C66" s="17" t="inlineStr">
+        <is>
+          <t>Wat is de verzuimfrequentie incl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D66" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E66" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F66" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="B67" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (in-/uitstroom)</t>
+        </is>
+      </c>
+      <c r="C67" s="17" t="inlineStr">
+        <is>
+          <t>Hoeveel zorgverleners in loondienst zijn er ingestroomd?</t>
+        </is>
+      </c>
+      <c r="D67" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E67" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F67" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="B68" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (in-/uitstroom)</t>
+        </is>
+      </c>
+      <c r="C68" s="17" t="inlineStr">
+        <is>
+          <t>Hoeveel zorgverleners in loondienst zijn er uitgestroomd?</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E68" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F68" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="B69" s="17" t="inlineStr">
+        <is>
+          <t>Personeel (in-/uitstroom)</t>
+        </is>
+      </c>
+      <c r="C69" s="17" t="inlineStr">
+        <is>
+          <t>Hoeveel personeel stroomt door naar een oplopend kwalificatieniveau?</t>
+        </is>
+      </c>
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E69" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F69" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="17" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="B70" s="17" t="inlineStr">
+        <is>
+          <t>Cliënten</t>
+        </is>
+      </c>
+      <c r="C70" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het aantal cliënten per zorgprofiel en vestiging?</t>
+        </is>
+      </c>
+      <c r="D70" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E70" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F70" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="B71" s="17" t="inlineStr">
+        <is>
+          <t>Cliënten</t>
+        </is>
+      </c>
+      <c r="C71" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het aantal cliënten per leveringsvorm met zorgprofiel VV?</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E71" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F71" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="17" t="inlineStr">
+        <is>
+          <t>14.3</t>
+        </is>
+      </c>
+      <c r="B72" s="17" t="inlineStr">
+        <is>
+          <t>Cliënten</t>
+        </is>
+      </c>
+      <c r="C72" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het aantal cliënten met een Wlz-indicatie per zorgprofiel VV en leveringsvorm?</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E72" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F72" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="inlineStr">
+        <is>
+          <t>16.1</t>
+        </is>
+      </c>
+      <c r="B73" s="17" t="inlineStr">
+        <is>
+          <t>Cliënten (Korsakov)</t>
+        </is>
+      </c>
+      <c r="C73" s="17" t="inlineStr">
+        <is>
+          <t>Hoeveel cliënten met het syndroom van Korsakov worden er verzorgd?</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E73" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F73" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:F73"/>
+  <mergeCells count="4">
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A4:F4"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId67"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F73"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Hardheidsclausule (beoordeling extra financiële middelen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Beoordeling welke gevalideerde vragen mogelijk bruikbaar zijn voor de hardheidsclausule: het beoordelingsproces of een</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>aanbieder in aanmerking komt voor extra financiële middelen bij zwaar weer. Afhankelijk van FTE, vastgoedcapaciteit en financiële data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Let op: dit is een inhoudelijke inschatting op basis van de vraagomschrijving, niet een officiële koppeling van Zilveren Kruis/KIK-V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Categorie</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Vraag (gevalideerde vraag)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Relevant?</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Onderbouwing</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Link naar indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het gemiddeld aantal personeelsleden?</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Directe FTE-/personeelsomvang-maatstaf (aantal medewerkers, ingezette/verloonde uren, contractomvang).</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het aantal personeelsleden?</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Directe FTE-/personeelsomvang-maatstaf (aantal medewerkers, ingezette/verloonde uren, contractomvang).</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Hoeveel uren zorggerelateerd personeel wordt ingezet?</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Directe FTE-/personeelsomvang-maatstaf (aantal medewerkers, ingezette/verloonde uren, contractomvang).</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Hoeveel uur zijn er verloond?</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Directe FTE-/personeelsomvang-maatstaf (aantal medewerkers, ingezette/verloonde uren, contractomvang).</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de gemiddelde contractomvang?</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Directe FTE-/personeelsomvang-maatstaf (aantal medewerkers, ingezette/verloonde uren, contractomvang).</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het aantal aanwezige wooneenheden?</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Vastgoedcapaciteit: aantal aanwezige/bezette wooneenheden en huisvestingscapaciteit per vestiging.</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>15.2</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het aantal bezette wooneenheden?</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Vastgoedcapaciteit: aantal aanwezige/bezette wooneenheden en huisvestingscapaciteit per vestiging.</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>15.3</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Hoeveel personen kunnen er per vestiging wonen?</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Vastgoedcapaciteit: aantal aanwezige/bezette wooneenheden en huisvestingscapaciteit per vestiging.</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>17.1.1</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal wooneenheden voor intramuraal en VPT geclusterd?</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Geplande toe-/afname van vastgoedcapaciteit (wooneenheden); direct relevant voor de vastgoedcapaciteit-component.</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>17.1.2</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal wooneenheden voor MPT en VPT niet-geclusterd?</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Geplande toe-/afname van vastgoedcapaciteit (wooneenheden); direct relevant voor de vastgoedcapaciteit-component.</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>18.1</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (balans / W&amp;V)</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de balans o.b.v. Grootboek?</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>18.2</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (balans / W&amp;V)</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de winst- en verliesrekening o.b.v. Grootboek?</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>19.1</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de DSCR (Debt Service Coverage Ratio)?</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>19.2</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is het werkkapitaal op korte termijn?</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>19.3</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de werkkapitaalratio?</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de quick ratio?</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>19.5</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de current ratio?</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>19.6</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de EBITDA (Earnings Before Interest, Tax, Deprecation and Amortisation)?</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de EBITDA-ratio?</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>19.8</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de cashflow?</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>20.1</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is de solvabiliteitsratio?</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>20.2</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is het weerstandsvermogen?</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>20.3</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is de debt ratio?</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat zijn de reserves?</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is de Reserves-Ratio?</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>21.1</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (rentabiliteit)</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>Rentabiliteit - wat is de winstratio?</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>21.2</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (rentabiliteit)</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>Rentabiliteit - wat is de REV (Resultaat Eigen Vermogen)?</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>22.1</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (groei)</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Groei - wat is de omzetgroei?</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>23.1</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (kapitaal)</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>Kapitaal - wat is de LTV (Loan to Value)?</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>23.2</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (kapitaal)</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>Kapitaal - wat is de net-debt / EBITDA?</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>23.3</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (kapitaal)</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>Kapitaal - wat is de CAPEX (Capital Expenditures)?</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>24.1</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de dekking van vaste activia door lang vermogen?</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>24.2</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de Interest Coverage Ratio (ICR)?</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>24.3</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de verhouding tussen kort en lang vreemd vermogen?</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>24.4</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de verhouding tussen vorderingen en opbrengsten?</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F41" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de arbeidsintensiteit PIL &amp; PNIL?</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>24.7</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is de arbeidsintensiteit PNIL?</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F43" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>24.9</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>Overig - wat is verhouding tussen uitbesteed werk en vast personeel?</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>Financiële kerncijfers/ratio (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal) rechtstreeks bruikbaar voor het inschatten van de financiële stabiliteit.</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Welk deel van de arbeidsovereenkomsten is voor bepaalde tijd?</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de leeftijdsopbouw van het personeel in loondienst?</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>Hoe zijn de ingezette uren zorgverleners verdeeld over de kwalificatieniveaus?</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F47" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het aantal ingezette uren zorgverleners in loondienst per cliënt?</t>
+        </is>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E48" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F48" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (PNIL)</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>Welk deel van de ingezette uren personeel is door PNIL?</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E49" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F49" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (PNIL)</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>Welk deel van de personeelskosten zijn voor PNIL?</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (vrijwilligers)</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het aantal vrijwilligers?</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E51" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F51" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (BBL)</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel BBL leerlingen zijn er?</t>
+        </is>
+      </c>
+      <c r="D52" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F52" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het kortdurend ziekteverzuimpercentage excl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D53" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F53" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het kortdurend ziekteverzuimpercentage incl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D54" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het langdurend ziekteverzuimpercentage excl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D55" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F55" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het langdurend ziekteverzuimpercentage incl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D56" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E56" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de verzuimfrequentie excl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D57" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F57" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C58" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de verzuimfrequentie incl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D58" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E58" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F58" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr">
+        <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (in-/uitstroom)</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel zorgverleners in loondienst zijn er ingestroomd?</t>
+        </is>
+      </c>
+      <c r="D59" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E59" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F59" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (in-/uitstroom)</t>
+        </is>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel zorgverleners in loondienst zijn er uitgestroomd?</t>
+        </is>
+      </c>
+      <c r="D60" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E60" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (in-/uitstroom)</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel personeel stroomt door naar een oplopend kwalificatieniveau?</t>
+        </is>
+      </c>
+      <c r="D61" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E61" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de FTE-inzet en personele kwetsbaarheid nader kan onderbouwen, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F61" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>15.4.1</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel cliënten met indicaties zijn er per financieringsstroom?</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E62" s="14" t="inlineStr">
+        <is>
+          <t>Financiële data over omzetsamenstelling (gedeclareerde bedragen per wet/sector); kan de financiële onderbouwing van de aanvraag ondersteunen.</t>
+        </is>
+      </c>
+      <c r="F62" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>15.4.2</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel Wlz-cliënten zijn er per sector?</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E63" s="14" t="inlineStr">
+        <is>
+          <t>Financiële data over omzetsamenstelling (gedeclareerde bedragen per wet/sector); kan de financiële onderbouwing van de aanvraag ondersteunen.</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>15.4.3</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel Wlz-cliënten met zorgprofiel VV zijn er per leveringsvorm?</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E64" s="14" t="inlineStr">
+        <is>
+          <t>Financiële data over omzetsamenstelling (gedeclareerde bedragen per wet/sector); kan de financiële onderbouwing van de aanvraag ondersteunen.</t>
+        </is>
+      </c>
+      <c r="F64" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t>15.4.4</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het gedeclareerde bedrag per wet?</t>
+        </is>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E65" s="14" t="inlineStr">
+        <is>
+          <t>Financiële data over omzetsamenstelling (gedeclareerde bedragen per wet/sector); kan de financiële onderbouwing van de aanvraag ondersteunen.</t>
+        </is>
+      </c>
+      <c r="F65" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>15.4.5</t>
+        </is>
+      </c>
+      <c r="B66" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het gedeclareerde bedrag per zorgsector?</t>
+        </is>
+      </c>
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E66" s="14" t="inlineStr">
+        <is>
+          <t>Financiële data over omzetsamenstelling (gedeclareerde bedragen per wet/sector); kan de financiële onderbouwing van de aanvraag ondersteunen.</t>
+        </is>
+      </c>
+      <c r="F66" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr">
+        <is>
+          <t>15.4.6</t>
+        </is>
+      </c>
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C67" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het gedeclareerde bedrag binnen Wlz-VV per leveringsvorm?</t>
+        </is>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E67" s="14" t="inlineStr">
+        <is>
+          <t>Financiële data over omzetsamenstelling (gedeclareerde bedragen per wet/sector); kan de financiële onderbouwing van de aanvraag ondersteunen.</t>
+        </is>
+      </c>
+      <c r="F67" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>17.2.1</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal cliënten voor intramuraal en VPT geclusterd?</t>
+        </is>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E68" s="14" t="inlineStr">
+        <is>
+          <t>Geplande cliëntontwikkeling gekoppeld aan de vastgoedplanning; indirect relevant voor de vastgoedcapaciteit-component.</t>
+        </is>
+      </c>
+      <c r="F68" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>17.2.2</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal cliënten voor MPT en VPT niet-geclusterd?</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E69" s="14" t="inlineStr">
+        <is>
+          <t>Geplande cliëntontwikkeling gekoppeld aan de vastgoedplanning; indirect relevant voor de vastgoedcapaciteit-component.</t>
+        </is>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="17" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="B70" s="17" t="inlineStr">
+        <is>
+          <t>Cliënten</t>
+        </is>
+      </c>
+      <c r="C70" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het aantal cliënten per zorgprofiel en vestiging?</t>
+        </is>
+      </c>
+      <c r="D70" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E70" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F70" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="B71" s="17" t="inlineStr">
+        <is>
+          <t>Cliënten</t>
+        </is>
+      </c>
+      <c r="C71" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het aantal cliënten per leveringsvorm met zorgprofiel VV?</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E71" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F71" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="17" t="inlineStr">
+        <is>
+          <t>14.3</t>
+        </is>
+      </c>
+      <c r="B72" s="17" t="inlineStr">
+        <is>
+          <t>Cliënten</t>
+        </is>
+      </c>
+      <c r="C72" s="17" t="inlineStr">
+        <is>
+          <t>Wat is het aantal cliënten met een Wlz-indicatie per zorgprofiel VV en leveringsvorm?</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E72" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F72" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="inlineStr">
+        <is>
+          <t>16.1</t>
+        </is>
+      </c>
+      <c r="B73" s="17" t="inlineStr">
+        <is>
+          <t>Cliënten (Korsakov)</t>
+        </is>
+      </c>
+      <c r="C73" s="17" t="inlineStr">
+        <is>
+          <t>Hoeveel cliënten met het syndroom van Korsakov worden er verzorgd?</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E73" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F73" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:F73"/>
+  <mergeCells count="4">
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A4:F4"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId67"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -3244,6 +7911,58 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Tabbladen 'EWS' en 'Hardheidsclausule':</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Deze tabbladen geven per gevalideerde vraag een inschatting (Ja / Mogelijk / Nee) of de vraag bruikbaar is voor het</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>betreffende proces, met een onderbouwing. Dit is een inhoudelijke inschatting op basis van de vraagomschrijving en</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>-categorie, GEEN officiële koppeling vanuit Zilveren Kruis of KIK-V. Controleer bij gebruik altijd de vraaginhoud zelf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>- Ja: de vraag levert direct bruikbare data voor het proces (FTE/vastgoedcapaciteit/financiële kerncijfers).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>- Mogelijk: de vraag levert ondersteunende/secundaire data die het proces kan onderbouwen, maar is geen kerngegeven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>- Nee: de vraag valt buiten de scope van het proces (bijv. cliëntgegevens die niet vastgoed/financieel/FTE betreffen).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Voeg Zorgkosten-sheet toe met relevantiebeoordeling
Beoordeling per gevalideerde vraag (Ja/Mogelijk/Nee, met onderbouwing)
of deze bruikbaar is voor het monitoren van zorgkosten van aanbieders,
op basis van informatie over capaciteit en FTE's.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HjW1Vn1BtW4ztesZ4qiQDe
</commit_message>
<xml_diff>
--- a/Gevalideerde_vragen_Uitwisselprofiel_Zorgkantoren.xlsx
+++ b/Gevalideerde_vragen_Uitwisselprofiel_Zorgkantoren.xlsx
@@ -10,12 +10,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gevalideerde vragen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EWS" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hardheidsclausule" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toelichting" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zorgkosten" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toelichting" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gevalideerde vragen'!$A$4:$G$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'EWS'!$A$6:$F$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hardheidsclausule'!$A$6:$F$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Zorgkosten'!$A$6:$F$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -7791,7 +7793,2309 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:F73"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Monitoren zorgkosten van aanbieders</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Beoordeling welke gevalideerde vragen mogelijk bruikbaar zijn voor het beoordelen/monitoren van zorgkosten van aanbieders,</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>waarbij gekeken wordt naar informatie over capaciteit en FTE's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Let op: dit is een inhoudelijke inschatting op basis van de vraagomschrijving, niet een officiële koppeling van Zilveren Kruis/KIK-V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Nr.</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Categorie</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Vraag (gevalideerde vraag)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Relevant?</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Onderbouwing</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Link naar indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het gemiddeld aantal personeelsleden?</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Directe FTE-maatstaf; nodig om zorgkosten te relateren aan personeelsinzet (bijv. kosten per FTE).</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het aantal personeelsleden?</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Directe FTE-maatstaf; nodig om zorgkosten te relateren aan personeelsinzet (bijv. kosten per FTE).</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Hoeveel uren zorggerelateerd personeel wordt ingezet?</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Directe FTE-maatstaf; nodig om zorgkosten te relateren aan personeelsinzet (bijv. kosten per FTE).</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Hoeveel uur zijn er verloond?</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Directe FTE-maatstaf; nodig om zorgkosten te relateren aan personeelsinzet (bijv. kosten per FTE).</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de gemiddelde contractomvang?</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Directe FTE-maatstaf; nodig om zorgkosten te relateren aan personeelsinzet (bijv. kosten per FTE).</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het aantal aanwezige wooneenheden?</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Vastgoedcapaciteit (aanwezige/bezette wooneenheden); nodig om zorgkosten te relateren aan capaciteitsbenutting (bijv. kosten per bezette plek).</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>15.2</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het aantal bezette wooneenheden?</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Vastgoedcapaciteit (aanwezige/bezette wooneenheden); nodig om zorgkosten te relateren aan capaciteitsbenutting (bijv. kosten per bezette plek).</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>15.3</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Hoeveel personen kunnen er per vestiging wonen?</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Vastgoedcapaciteit (aanwezige/bezette wooneenheden); nodig om zorgkosten te relateren aan capaciteitsbenutting (bijv. kosten per bezette plek).</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>15.4.4</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het gedeclareerde bedrag per wet?</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Betreft de zorgkosten zelf (gedeclareerd bedrag per wet/zorgsector/leveringsvorm) — kernindicator voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>15.4.5</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het gedeclareerde bedrag per zorgsector?</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Betreft de zorgkosten zelf (gedeclareerd bedrag per wet/zorgsector/leveringsvorm) — kernindicator voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>15.4.6</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Wat is het gedeclareerde bedrag binnen Wlz-VV per leveringsvorm?</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Betreft de zorgkosten zelf (gedeclareerd bedrag per wet/zorgsector/leveringsvorm) — kernindicator voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>17.1.1</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal wooneenheden voor intramuraal en VPT geclusterd?</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Geplande capaciteitsuitbreiding/-afbouw (wooneenheden); relevant voor de toekomstige verhouding tussen capaciteit en zorgkosten.</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>17.1.2</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal wooneenheden voor MPT en VPT niet-geclusterd?</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Geplande capaciteitsuitbreiding/-afbouw (wooneenheden); relevant voor de toekomstige verhouding tussen capaciteit en zorgkosten.</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Welk deel van de arbeidsovereenkomsten is voor bepaalde tijd?</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de leeftijdsopbouw van het personeel in loondienst?</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>Hoe zijn de ingezette uren zorgverleners verdeeld over de kwalificatieniveaus?</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Personeel</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het aantal ingezette uren zorgverleners in loondienst per cliënt?</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (PNIL)</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Welk deel van de ingezette uren personeel is door PNIL?</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (PNIL)</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Welk deel van de personeelskosten zijn voor PNIL?</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (vrijwilligers)</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het aantal vrijwilligers?</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (BBL)</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel BBL leerlingen zijn er?</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het kortdurend ziekteverzuimpercentage excl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het kortdurend ziekteverzuimpercentage incl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F29" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het langdurend ziekteverzuimpercentage excl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>11.4</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het langdurend ziekteverzuimpercentage incl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>12.1</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de verzuimfrequentie excl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (verzuim)</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de verzuimfrequentie incl. zwangerschapsverlof?</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>13.1</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (in-/uitstroom)</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel zorgverleners in loondienst zijn er ingestroomd?</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F34" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>13.2</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (in-/uitstroom)</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel zorgverleners in loondienst zijn er uitgestroomd?</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F35" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>13.3</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>Personeel (in-/uitstroom)</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel personeel stroomt door naar een oplopend kwalificatieniveau?</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>Aanvullende personeelsindicator (samenstelling, verzuim, in-/uitstroom, PNIL-aandeel) die de personeelsinzet nader onderbouwt bij het duiden van zorgkosten, maar is zelf geen directe FTE-maatstaf.</t>
+        </is>
+      </c>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>14.1</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>Cliënten</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het aantal cliënten per zorgprofiel en vestiging?</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>Aantal cliënten per zorgprofiel/leveringsvorm/vestiging; nodig als noemer voor kosten-per-cliënt-analyses en om bezetting aan zorgkosten te relateren.</t>
+        </is>
+      </c>
+      <c r="F37" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>14.2</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Cliënten</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het aantal cliënten per leveringsvorm met zorgprofiel VV?</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>Aantal cliënten per zorgprofiel/leveringsvorm/vestiging; nodig als noemer voor kosten-per-cliënt-analyses en om bezetting aan zorgkosten te relateren.</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>14.3</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>Cliënten</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>Wat is het aantal cliënten met een Wlz-indicatie per zorgprofiel VV en leveringsvorm?</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>Aantal cliënten per zorgprofiel/leveringsvorm/vestiging; nodig als noemer voor kosten-per-cliënt-analyses en om bezetting aan zorgkosten te relateren.</t>
+        </is>
+      </c>
+      <c r="F39" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>15.4.1</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel cliënten met indicaties zijn er per financieringsstroom?</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>Volume-informatie (cliënten per financieringsstroom/sector/leveringsvorm) die de omvang van de zorgkosten mede verklaart.</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>15.4.2</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel Wlz-cliënten zijn er per sector?</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>Volume-informatie (cliënten per financieringsstroom/sector/leveringsvorm) die de omvang van de zorgkosten mede verklaart.</t>
+        </is>
+      </c>
+      <c r="F41" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>15.4.3</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteit / wooneenheden / Wlz-financiering</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel Wlz-cliënten met zorgprofiel VV zijn er per leveringsvorm?</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>Volume-informatie (cliënten per financieringsstroom/sector/leveringsvorm) die de omvang van de zorgkosten mede verklaart.</t>
+        </is>
+      </c>
+      <c r="F42" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>16.1</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>Cliënten (Korsakov)</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>Hoeveel cliënten met het syndroom van Korsakov worden er verzorgd?</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>Cliëntenaantal voor een specifieke, kostenintensieve doelgroep (Korsakov); kan relevant zijn bij het duiden van zorgkosten voor deze groep.</t>
+        </is>
+      </c>
+      <c r="F43" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>17.2.1</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal cliënten voor intramuraal en VPT geclusterd?</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>Geplande cliëntontwikkeling gekoppeld aan de vastgoedplanning; indirect relevant voor toekomstige zorgkosten per cliënt.</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>17.2.2</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Capaciteitsplanning</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Wat is de geplande toe- en afname van het aantal cliënten voor MPT en VPT niet-geclusterd?</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>Mogelijk</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>Geplande cliëntontwikkeling gekoppeld aan de vastgoedplanning; indirect relevant voor toekomstige zorgkosten per cliënt.</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>18.1</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (balans / W&amp;V)</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>Wat is de balans o.b.v. Grootboek?</t>
+        </is>
+      </c>
+      <c r="D46" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E46" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F46" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>18.2</t>
+        </is>
+      </c>
+      <c r="B47" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (balans / W&amp;V)</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>Wat is de winst- en verliesrekening o.b.v. Grootboek?</t>
+        </is>
+      </c>
+      <c r="D47" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F47" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>19.1</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de DSCR (Debt Service Coverage Ratio)?</t>
+        </is>
+      </c>
+      <c r="D48" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E48" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F48" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>19.2</t>
+        </is>
+      </c>
+      <c r="B49" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is het werkkapitaal op korte termijn?</t>
+        </is>
+      </c>
+      <c r="D49" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F49" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>19.3</t>
+        </is>
+      </c>
+      <c r="B50" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de werkkapitaalratio?</t>
+        </is>
+      </c>
+      <c r="D50" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E50" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F50" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>19.4</t>
+        </is>
+      </c>
+      <c r="B51" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de quick ratio?</t>
+        </is>
+      </c>
+      <c r="D51" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E51" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F51" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>19.5</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de current ratio?</t>
+        </is>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F52" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>19.6</t>
+        </is>
+      </c>
+      <c r="B53" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de EBITDA (Earnings Before Interest, Tax, Deprecation and Amortisation)?</t>
+        </is>
+      </c>
+      <c r="D53" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F53" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de EBITDA-ratio?</t>
+        </is>
+      </c>
+      <c r="D54" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F54" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>19.8</t>
+        </is>
+      </c>
+      <c r="B55" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (liquiditeit)</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="inlineStr">
+        <is>
+          <t>Liquiditeit - wat is de cashflow?</t>
+        </is>
+      </c>
+      <c r="D55" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F55" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>20.1</t>
+        </is>
+      </c>
+      <c r="B56" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C56" s="17" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is de solvabiliteitsratio?</t>
+        </is>
+      </c>
+      <c r="D56" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F56" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>20.2</t>
+        </is>
+      </c>
+      <c r="B57" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C57" s="17" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is het weerstandsvermogen?</t>
+        </is>
+      </c>
+      <c r="D57" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E57" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F57" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t>20.3</t>
+        </is>
+      </c>
+      <c r="B58" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C58" s="17" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is de debt ratio?</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E58" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F58" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>20.4</t>
+        </is>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat zijn de reserves?</t>
+        </is>
+      </c>
+      <c r="D59" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E59" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F59" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="B60" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (solvabiliteit)</t>
+        </is>
+      </c>
+      <c r="C60" s="17" t="inlineStr">
+        <is>
+          <t>Solvabiliteit - wat is de Reserves-Ratio?</t>
+        </is>
+      </c>
+      <c r="D60" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E60" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F60" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>21.1</t>
+        </is>
+      </c>
+      <c r="B61" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (rentabiliteit)</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="inlineStr">
+        <is>
+          <t>Rentabiliteit - wat is de winstratio?</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E61" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F61" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>21.2</t>
+        </is>
+      </c>
+      <c r="B62" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (rentabiliteit)</t>
+        </is>
+      </c>
+      <c r="C62" s="17" t="inlineStr">
+        <is>
+          <t>Rentabiliteit - wat is de REV (Resultaat Eigen Vermogen)?</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E62" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F62" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>22.1</t>
+        </is>
+      </c>
+      <c r="B63" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (groei)</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>Groei - wat is de omzetgroei?</t>
+        </is>
+      </c>
+      <c r="D63" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E63" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F63" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t>23.1</t>
+        </is>
+      </c>
+      <c r="B64" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (kapitaal)</t>
+        </is>
+      </c>
+      <c r="C64" s="17" t="inlineStr">
+        <is>
+          <t>Kapitaal - wat is de LTV (Loan to Value)?</t>
+        </is>
+      </c>
+      <c r="D64" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E64" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F64" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>23.2</t>
+        </is>
+      </c>
+      <c r="B65" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (kapitaal)</t>
+        </is>
+      </c>
+      <c r="C65" s="17" t="inlineStr">
+        <is>
+          <t>Kapitaal - wat is de net-debt / EBITDA?</t>
+        </is>
+      </c>
+      <c r="D65" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E65" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F65" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>23.3</t>
+        </is>
+      </c>
+      <c r="B66" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (kapitaal)</t>
+        </is>
+      </c>
+      <c r="C66" s="17" t="inlineStr">
+        <is>
+          <t>Kapitaal - wat is de CAPEX (Capital Expenditures)?</t>
+        </is>
+      </c>
+      <c r="D66" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E66" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F66" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>24.1</t>
+        </is>
+      </c>
+      <c r="B67" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C67" s="17" t="inlineStr">
+        <is>
+          <t>Overig - wat is de dekking van vaste activia door lang vermogen?</t>
+        </is>
+      </c>
+      <c r="D67" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E67" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F67" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t>24.2</t>
+        </is>
+      </c>
+      <c r="B68" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C68" s="17" t="inlineStr">
+        <is>
+          <t>Overig - wat is de Interest Coverage Ratio (ICR)?</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E68" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F68" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>24.3</t>
+        </is>
+      </c>
+      <c r="B69" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C69" s="17" t="inlineStr">
+        <is>
+          <t>Overig - wat is de verhouding tussen kort en lang vreemd vermogen?</t>
+        </is>
+      </c>
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E69" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F69" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="17" t="inlineStr">
+        <is>
+          <t>24.4</t>
+        </is>
+      </c>
+      <c r="B70" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C70" s="17" t="inlineStr">
+        <is>
+          <t>Overig - wat is de verhouding tussen vorderingen en opbrengsten?</t>
+        </is>
+      </c>
+      <c r="D70" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E70" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F70" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>24.5</t>
+        </is>
+      </c>
+      <c r="B71" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C71" s="17" t="inlineStr">
+        <is>
+          <t>Overig - wat is de arbeidsintensiteit PIL &amp; PNIL?</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E71" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F71" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="17" t="inlineStr">
+        <is>
+          <t>24.7</t>
+        </is>
+      </c>
+      <c r="B72" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C72" s="17" t="inlineStr">
+        <is>
+          <t>Overig - wat is de arbeidsintensiteit PNIL?</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E72" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F72" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="inlineStr">
+        <is>
+          <t>24.9</t>
+        </is>
+      </c>
+      <c r="B73" s="17" t="inlineStr">
+        <is>
+          <t>Financieel (overig)</t>
+        </is>
+      </c>
+      <c r="C73" s="17" t="inlineStr">
+        <is>
+          <t>Overig - wat is verhouding tussen uitbesteed werk en vast personeel?</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="E73" s="17" t="inlineStr">
+        <is>
+          <t>Betreft brede financiële stabiliteitsratio's (balans, liquiditeit, solvabiliteit, rentabiliteit, groei, kapitaal), niet specifiek capaciteit- of FTE-gerelateerd; buiten de scope zoals aangegeven voor dit proces.</t>
+        </is>
+      </c>
+      <c r="F73" s="19" t="inlineStr">
+        <is>
+          <t>Bekijk indicator</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:F73"/>
+  <mergeCells count="4">
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A4:F4"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId67"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -7963,6 +10267,37 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Tabblad 'Zorgkosten':</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Beoordeling welke vragen bruikbaar zijn voor het monitoren van zorgkosten van aanbieders, waarbij gekeken wordt naar</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>informatie over capaciteit (wooneenheden, gedeclareerde bedragen) en FTE's. Zelfde Ja/Mogelijk/Nee-systematiek als bij</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>de tabbladen EWS en Hardheidsclausule.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>